<commit_message>
Fix safety stock formula & clarify stock coverage term
- Safety stock now uses the transparent model SS = Z * lead-time demand * variability
  (1.28 * 0.5 * 0.3 * monthly demand), readable and interview-friendly.
- Rename 'stock_turn' -> 'stock_coverage' to avoid confusion with the annual
  inventory-turnover ratio; it means months of demand covered.
- Regenerate output tables and figure.
</commit_message>
<xml_diff>
--- a/output/inventory_optimization_result.xlsx
+++ b/output/inventory_optimization_result.xlsx
@@ -444,7 +444,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>stock_turn</t>
+          <t>stock_coverage</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -478,7 +478,7 @@
         <v>1750</v>
       </c>
       <c r="E2" t="n">
-        <v>244</v>
+        <v>173</v>
       </c>
       <c r="F2" t="n">
         <v>1.94</v>
@@ -512,7 +512,7 @@
         <v>820</v>
       </c>
       <c r="E3" t="n">
-        <v>407</v>
+        <v>288</v>
       </c>
       <c r="F3" t="n">
         <v>0.55</v>
@@ -546,7 +546,7 @@
         <v>960</v>
       </c>
       <c r="E4" t="n">
-        <v>190</v>
+        <v>134</v>
       </c>
       <c r="F4" t="n">
         <v>1.37</v>
@@ -580,7 +580,7 @@
         <v>120</v>
       </c>
       <c r="E5" t="n">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="F5" t="n">
         <v>0.48</v>
@@ -614,7 +614,7 @@
         <v>300</v>
       </c>
       <c r="E6" t="n">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="F6" t="n">
         <v>0.86</v>
@@ -648,7 +648,7 @@
         <v>1500</v>
       </c>
       <c r="E7" t="n">
-        <v>299</v>
+        <v>211</v>
       </c>
       <c r="F7" t="n">
         <v>1.36</v>
@@ -682,7 +682,7 @@
         <v>2400</v>
       </c>
       <c r="E8" t="n">
-        <v>597</v>
+        <v>422</v>
       </c>
       <c r="F8" t="n">
         <v>1.09</v>
@@ -716,7 +716,7 @@
         <v>410</v>
       </c>
       <c r="E9" t="n">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="F9" t="n">
         <v>1.71</v>
@@ -750,7 +750,7 @@
         <v>400</v>
       </c>
       <c r="E10" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="F10" t="n">
         <v>2.22</v>
@@ -784,7 +784,7 @@
         <v>780</v>
       </c>
       <c r="E11" t="n">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="F11" t="n">
         <v>1.5</v>
@@ -818,7 +818,7 @@
         <v>560</v>
       </c>
       <c r="E12" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="F12" t="n">
         <v>1.87</v>
@@ -852,7 +852,7 @@
         <v>3200</v>
       </c>
       <c r="E13" t="n">
-        <v>760</v>
+        <v>538</v>
       </c>
       <c r="F13" t="n">
         <v>1.14</v>

</xml_diff>